<commit_message>
docs(aidlc): add prompt-cache/context-reuse metrics to ACU report and workbook
Co-Authored-By: samrat.kar@infosys.com <samrat.kar@infosys.com>
</commit_message>
<xml_diff>
--- a/docs/migration/aidlc-acu-metrics.xlsx
+++ b/docs/migration/aidlc-acu-metrics.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACU Cost" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt cache" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -85,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,6 +112,12 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1294,4 +1302,975 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt cache / context reuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Devin bills in ACUs and does not price prompt cache separately, nor expose Claude cache_read_input_tokens/cache_creation_input_tokens. These figures are derived from the session's context_growth_update telemetry (current_context_tokens per agent iteration): the stable prefix re-sent on iteration N (= context size at N-1) is what a prompt cache serves as a cache read, and the delta is newly written cache.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Source: context_growth_update events (41 samples, iterations 1-59), linearly interpolated between samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Iterations</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Prompt tokens processed</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Cache-read tokens</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Cache-creation tokens</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Cache hit rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Measured window</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1-59</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>4687264</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>4583352</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>103912</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>0.978</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Full session (extrapolated)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>1-150</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>19136288</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>18923832</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>212456</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>0.9890000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Agent iteration</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Context tokens</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Cache-read tokens</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Cache-creation tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>34730</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>34730</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>38863</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>34730</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>4133</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>44822</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>38863</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>5959</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>44822</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>53798</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>7473</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>54348</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>53798</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>57223</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>54348</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>2875</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>58063</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>57223</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>62634</v>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>58063</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>65242</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>62634</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>2608</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>66137</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>65242</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>67274</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>66137</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" s="15" t="n">
+        <v>67830</v>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>67274</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>68386</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>67830</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>69055</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>68386</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>69586</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>69055</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>70802</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>69586</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>72047</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>70802</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>72476</v>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>72047</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>72904</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>72476</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>73986</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>72904</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>74575</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>73986</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>75164</v>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>74575</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>76604</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>75164</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>77318</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>76604</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>78033</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>77318</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>78564</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>78033</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>79094</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>78564</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="15" t="n">
+        <v>80170</v>
+      </c>
+      <c r="C38" s="15" t="n">
+        <v>79094</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="15" t="n">
+        <v>81246</v>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>80170</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="B40" s="15" t="n">
+        <v>81757</v>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>81246</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>82268</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>81757</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="n">
+        <v>33</v>
+      </c>
+      <c r="B42" s="15" t="n">
+        <v>83363</v>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>82268</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="n">
+        <v>34</v>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>83940</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>83363</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="B44" s="15" t="n">
+        <v>84516</v>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>83940</v>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>86140</v>
+      </c>
+      <c r="C45" s="15" t="n">
+        <v>84516</v>
+      </c>
+      <c r="D45" s="15" t="n">
+        <v>1624</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
+        <v>37</v>
+      </c>
+      <c r="B46" s="15" t="n">
+        <v>86840</v>
+      </c>
+      <c r="C46" s="15" t="n">
+        <v>86140</v>
+      </c>
+      <c r="D46" s="15" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="n">
+        <v>38</v>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>87540</v>
+      </c>
+      <c r="C47" s="15" t="n">
+        <v>86840</v>
+      </c>
+      <c r="D47" s="15" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="n">
+        <v>39</v>
+      </c>
+      <c r="B48" s="15" t="n">
+        <v>87902</v>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>87540</v>
+      </c>
+      <c r="D48" s="15" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>88264</v>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>87902</v>
+      </c>
+      <c r="D49" s="15" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" s="15" t="n">
+        <v>89157</v>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>88264</v>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="B51" s="15" t="n">
+        <v>90050</v>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>89157</v>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="n">
+        <v>43</v>
+      </c>
+      <c r="B52" s="15" t="n">
+        <v>92004</v>
+      </c>
+      <c r="C52" s="15" t="n">
+        <v>90050</v>
+      </c>
+      <c r="D52" s="15" t="n">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="n">
+        <v>44</v>
+      </c>
+      <c r="B53" s="15" t="n">
+        <v>92625</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>92004</v>
+      </c>
+      <c r="D53" s="15" t="n">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B54" s="15" t="n">
+        <v>93247</v>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>92625</v>
+      </c>
+      <c r="D54" s="15" t="n">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="n">
+        <v>46</v>
+      </c>
+      <c r="B55" s="15" t="n">
+        <v>93868</v>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>93247</v>
+      </c>
+      <c r="D55" s="15" t="n">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" s="15" t="n">
+        <v>94508</v>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>93868</v>
+      </c>
+      <c r="D56" s="15" t="n">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" s="15" t="n">
+        <v>95507</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <v>94508</v>
+      </c>
+      <c r="D57" s="15" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="B58" s="15" t="n">
+        <v>96324</v>
+      </c>
+      <c r="C58" s="15" t="n">
+        <v>95507</v>
+      </c>
+      <c r="D58" s="15" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="B59" s="15" t="n">
+        <v>97140</v>
+      </c>
+      <c r="C59" s="15" t="n">
+        <v>96324</v>
+      </c>
+      <c r="D59" s="15" t="n">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="n">
+        <v>51</v>
+      </c>
+      <c r="B60" s="15" t="n">
+        <v>98496</v>
+      </c>
+      <c r="C60" s="15" t="n">
+        <v>97140</v>
+      </c>
+      <c r="D60" s="15" t="n">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="n">
+        <v>52</v>
+      </c>
+      <c r="B61" s="15" t="n">
+        <v>99373</v>
+      </c>
+      <c r="C61" s="15" t="n">
+        <v>98496</v>
+      </c>
+      <c r="D61" s="15" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="n">
+        <v>53</v>
+      </c>
+      <c r="B62" s="15" t="n">
+        <v>100250</v>
+      </c>
+      <c r="C62" s="15" t="n">
+        <v>99373</v>
+      </c>
+      <c r="D62" s="15" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="n">
+        <v>54</v>
+      </c>
+      <c r="B63" s="15" t="n">
+        <v>101127</v>
+      </c>
+      <c r="C63" s="15" t="n">
+        <v>100250</v>
+      </c>
+      <c r="D63" s="15" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="B64" s="15" t="n">
+        <v>101462</v>
+      </c>
+      <c r="C64" s="15" t="n">
+        <v>101127</v>
+      </c>
+      <c r="D64" s="15" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="n">
+        <v>56</v>
+      </c>
+      <c r="B65" s="15" t="n">
+        <v>102156</v>
+      </c>
+      <c r="C65" s="15" t="n">
+        <v>101462</v>
+      </c>
+      <c r="D65" s="15" t="n">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="B66" s="15" t="n">
+        <v>102850</v>
+      </c>
+      <c r="C66" s="15" t="n">
+        <v>102156</v>
+      </c>
+      <c r="D66" s="15" t="n">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="n">
+        <v>58</v>
+      </c>
+      <c r="B67" s="15" t="n">
+        <v>103381</v>
+      </c>
+      <c r="C67" s="15" t="n">
+        <v>102850</v>
+      </c>
+      <c r="D67" s="15" t="n">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="B68" s="15" t="n">
+        <v>103912</v>
+      </c>
+      <c r="C68" s="15" t="n">
+        <v>103381</v>
+      </c>
+      <c r="D68" s="15" t="n">
+        <v>531</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>